<commit_message>
feat: implement dummy profiles switcher, real-time checklist approvals, WBS scroll, and workspace linter fix
</commit_message>
<xml_diff>
--- a/PMO_Weekly_Report_Data.xlsx
+++ b/PMO_Weekly_Report_Data.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NextSteps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approvals" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,48 +430,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Planned %</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Actual %</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Actual Cost</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Delay Days</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Approved By</t>
         </is>
       </c>
     </row>
@@ -491,6 +509,11 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Mike Johnson (Project Manager)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -521,96 +544,69 @@
       <c r="H3" t="n">
         <v>2</v>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beone</t>
+          <t>redone</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Charlie</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="E4" t="n">
-        <v>35000</v>
+        <v>120000</v>
       </c>
       <c r="F4" t="n">
-        <v>36000</v>
+        <v>115000</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>redone</t>
+          <t>tuntalk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E5" t="n">
-        <v>120000</v>
+        <v>45000</v>
       </c>
       <c r="F5" t="n">
-        <v>115000</v>
+        <v>48000</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Ethan</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>40</v>
-      </c>
-      <c r="D6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E6" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>48000</v>
-      </c>
-      <c r="G6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H6" t="n">
         <v>4</v>
       </c>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -623,16 +619,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Achievement</t>
         </is>
@@ -665,34 +661,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beone</t>
+          <t>redone</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Initial stakeholder requirements gathering phase completed.</t>
+          <t>Phase 1 user acceptance testing successfully concluded.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>redone</t>
+          <t>tuntalk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>Phase 1 user acceptance testing successfully concluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
         <is>
           <t>Vendor integration contracts finalized and signed.</t>
         </is>
@@ -709,31 +693,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Risk Description</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Mitigation</t>
         </is>
@@ -742,17 +726,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Beone</t>
+          <t>tuntalk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Resource constraints in development team</t>
+          <t>API documentation delays from vendor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -761,33 +745,6 @@
         </is>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>Onboard contract resources to plug skill gaps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>API documentation delays from vendor</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>Escalate to vendor management and setup daily syncs.</t>
         </is>
@@ -804,26 +761,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
@@ -876,64 +833,42 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Beone</t>
+          <t>redone</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Draft formal functional specifications document</t>
+          <t>Initiate Phase 2 frontend development modules</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Charlie</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>redone</t>
+          <t>tuntalk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Initiate Phase 2 frontend development modules</t>
+          <t>Establish connection sandbox with vendor gateways</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Establish connection sandbox with vendor gateways</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Ethan</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
@@ -950,31 +885,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Decision Required</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -983,54 +918,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Beone</t>
+          <t>tuntalk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Approve additional budget for contractors</t>
+          <t>Select alternative API gateway vendor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Needed to keep requirement phase on schedule.</t>
+          <t>Current vendor is unresponsive on SLA terms.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Approve / Reject</t>
+          <t>Vendor A / Vendor B</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Approve and source from PMO buffer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Select alternative API gateway vendor</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Current vendor is unresponsive on SLA terms.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Vendor A / Vendor B</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>Migrate to Vendor B immediately.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Approved By</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Approved Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-15 23:59:10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mike Johnson (Project Manager)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>freedom</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement Project Scope registry and Excel database synchronization
</commit_message>
<xml_diff>
--- a/PMO_Weekly_Report_Data.xlsx
+++ b/PMO_Weekly_Report_Data.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NextSteps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approvals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProjectScope" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approvals" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -953,29 +954,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Approved By</t>
+          <t>Pre-sales Document</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Approved Projects</t>
+          <t>Pre-sales Scope Prepare</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pre-sales Project Time Plan</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Risk Register Party Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Presentation Kick Off</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Presentation Weekly</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Presentation Monthly</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Internal Reports Presentation Format</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Project Progress</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>freedom</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Test Doc 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Test Scope 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Test Plan 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Test Party 1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Test Kickoff 1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Test Weekly 1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Test Monthly 1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Test Format 1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Test Progress 1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Approved By</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Approved Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>2026-06-15 23:59:10</t>
         </is>
       </c>
@@ -989,6 +1108,32 @@
           <t>freedom</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:18:20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:29:02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Redesign Project Scope registry into 6-step wizard and implement dual pre-sales and agreed doc upload ingestion
</commit_message>
<xml_diff>
--- a/PMO_Weekly_Report_Data.xlsx
+++ b/PMO_Weekly_Report_Data.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,25 +484,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>freedom</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>elena</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="F2" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -512,102 +512,9 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>John Doe (PMO Lead)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ATT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Bob</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>70</v>
-      </c>
-      <c r="D3" t="n">
-        <v>65</v>
-      </c>
-      <c r="E3" t="n">
-        <v>80000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>78000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>redone</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Diana</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>90</v>
-      </c>
-      <c r="D4" t="n">
-        <v>90</v>
-      </c>
-      <c r="E4" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>115000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ethan</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>40</v>
-      </c>
-      <c r="D5" t="n">
-        <v>30</v>
-      </c>
-      <c r="E5" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>48000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>Alex Marques (Head of PMO)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -620,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,54 +539,6 @@
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Achievement</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>freedom</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Project charter approved and kickoff completed successfully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ATT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Staging environment configuration finalized and verified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>redone</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Phase 1 user acceptance testing successfully concluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Vendor integration contracts finalized and signed.</t>
         </is>
       </c>
     </row>
@@ -694,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,33 +580,6 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Mitigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>API documentation delays from vendor</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Escalate to vendor management and setup daily syncs.</t>
         </is>
       </c>
     </row>
@@ -762,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -784,94 +616,6 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Deadline</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>freedom</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Setup Git repository and configure CI/CD pipeline</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Alex</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ATT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Deploy initial sandbox build for security review</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Bob</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>redone</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Initiate Phase 2 frontend development modules</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Diana</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Establish connection sandbox with vendor gateways</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Ethan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -886,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -913,33 +657,6 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Recommendation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>tuntalk</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Select alternative API gateway vendor</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Current vendor is unresponsive on SLA terms.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Vendor A / Vendor B</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Migrate to Vendor B immediately.</t>
         </is>
       </c>
     </row>
@@ -1072,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1135,6 +852,71 @@
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-27 18:01:10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-27 18:01:12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-27 18:01:15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-27 18:01:17</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-27 18:06:06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Agreed Document and Risk Register tabs from Project Scope wizard
</commit_message>
<xml_diff>
--- a/PMO_Weekly_Report_Data.xlsx
+++ b/PMO_Weekly_Report_Data.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vivo</t>
+          <t>freedom</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -510,11 +510,7 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Alex Marques (Head of PMO)</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -671,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,42 +683,82 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pre-sales Scope Prepare</t>
+          <t>Components</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Pre-sales Project Time Plan</t>
+          <t>Scope Prepare</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Project Time Plan</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Agreed Document</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Project Plan</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Scope In</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Scope Out</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Presentation Type</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Kick Off</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Milestone Progress</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Project Status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Status</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Executive Presentation</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Risk Register Party Expected</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Customer Presentation Kick Off</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Customer Presentation Weekly</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Customer Presentation Monthly</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Internal Reports Presentation Format</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Project Progress</t>
         </is>
       </c>
     </row>
@@ -737,44 +773,24 @@
           <t>Test Doc 1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Test Scope 1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Test Plan 1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Test Party 1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Test Kickoff 1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Test Weekly 1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Test Monthly 1</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Test Format 1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Test Progress 1</t>
         </is>
       </c>
     </row>
@@ -789,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -917,6 +933,19 @@
       </c>
       <c r="C9" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:16:09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>